<commit_message>
fix(job-19a): SNOMED 對照表逐筆覆核並閘門化 loinc_preferred 一致性
JOB-19 線 A（SNOMED 對映覆核；線 B UCUM 稽核另一 PR）。方向：以值集為真、
重建衍生資產，不得以 CSV 回填值集。

snomed-loinc-mappings.csv（33 列）逐筆比對 loinc_preferred 與 IG 值集成員：
- 視力 Panel：79880-1（單眼最佳矯正 Snellen，語意錯）→ 98497-1（IG 實際採用之
  Visual acuity panel）。
- 腰臀比 WHR：73708-3（tx 驗證為無效碼，已自值集移除）→ 「(-確定無合適碼)」哨符。
- snomed_status：33 列全數 VERIFIED → 待覆核。§4.1 唯一之 SNOMED $validate-code
  覆核（4 個社會史/服務碼）不涵蓋本 CSV 之實驗室對映碼，故無一符合保留 VERIFIED
  之條件（不得因 LOINC 側對了就標 VERIFIED——正是四度出錯之成因）。

閘門化：新增 scripts/check-asset-consistency.js，驗證每個非哨符 loinc_preferred
存在於某 IG 值集，納入 npm run check:assets。負向測試：改為值集外之碼即失敗。

未變更任何值集內容（VS-ExtendedDataset 維持 288）。snomed-mappings.xlsx 隨 CSV 重建。
逐筆紀錄見 docs/optimization/evidence/job-19-line-a-snomed-reconciliation.md。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjF2Z8BacRouh49x56vfaA
</commit_message>
<xml_diff>
--- a/input/assets/snomed-mappings.xlsx
+++ b/input/assets/snomed-mappings.xlsx
@@ -295,7 +295,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -343,7 +343,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I25"/>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I26"/>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I27"/>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">73708-3</t>
+          <t xml:space="preserve">(-確定無合適碼)</t>
         </is>
       </c>
       <c r="E29"/>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I30"/>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">79880-1</t>
+          <t xml:space="preserve">98497-1</t>
         </is>
       </c>
       <c r="E33"/>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I33"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">

</xml_diff>